<commit_message>
Added selected 4 folders
</commit_message>
<xml_diff>
--- a/Excel data cleaning/product_category_name_translation.xlsx
+++ b/Excel data cleaning/product_category_name_translation.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/9cb9f3fc979f0a51/Desktop/Final Project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="22" documentId="8_{1255C78C-4A46-4BA2-98C7-D840E1B35E98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A4159E83-1046-41BF-AA12-C9E99A97069E}"/>
+  <xr:revisionPtr revIDLastSave="25" documentId="8_{1255C78C-4A46-4BA2-98C7-D840E1B35E98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DCB8FDA4-271B-4632-9904-58FDE221D498}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{9D35D31A-0E0E-4CA1-A58D-180E2C0E804E}"/>
   </bookViews>
@@ -1325,9 +1325,9 @@
         <f>PROPER(TRIM(A1))</f>
         <v>Product_Category_Name</v>
       </c>
-      <c r="D1" t="str">
-        <f>PROPER(TRIM(B1))</f>
-        <v>Product_Category_Name_English</v>
+      <c r="D1">
+        <f>H9</f>
+        <v>0</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
@@ -1338,11 +1338,11 @@
         <v>3</v>
       </c>
       <c r="C2" t="str">
-        <f t="shared" ref="C2:C65" si="0">PROPER(TRIM(A2))</f>
+        <f>PROPER(TRIM(A2))</f>
         <v>Beleza_Saude</v>
       </c>
       <c r="D2" t="str">
-        <f t="shared" ref="D2:D65" si="1">PROPER(TRIM(B2))</f>
+        <f>PROPER(TRIM(B2))</f>
         <v>Health_Beauty</v>
       </c>
     </row>
@@ -1354,11 +1354,11 @@
         <v>5</v>
       </c>
       <c r="C3" t="str">
-        <f t="shared" si="0"/>
+        <f>PROPER(TRIM(A3))</f>
         <v>Informatica_Acessorios</v>
       </c>
       <c r="D3" t="str">
-        <f t="shared" si="1"/>
+        <f>PROPER(TRIM(B3))</f>
         <v>Computers_Accessories</v>
       </c>
     </row>
@@ -1370,11 +1370,11 @@
         <v>7</v>
       </c>
       <c r="C4" t="str">
-        <f t="shared" si="0"/>
+        <f>PROPER(TRIM(A4))</f>
         <v>Automotivo</v>
       </c>
       <c r="D4" t="str">
-        <f t="shared" si="1"/>
+        <f>PROPER(TRIM(B4))</f>
         <v>Auto</v>
       </c>
     </row>
@@ -1386,11 +1386,11 @@
         <v>9</v>
       </c>
       <c r="C5" t="str">
-        <f t="shared" si="0"/>
+        <f>PROPER(TRIM(A5))</f>
         <v>Cama_Mesa_Banho</v>
       </c>
       <c r="D5" t="str">
-        <f t="shared" si="1"/>
+        <f>PROPER(TRIM(B5))</f>
         <v>Bed_Bath_Table</v>
       </c>
     </row>
@@ -1402,11 +1402,11 @@
         <v>11</v>
       </c>
       <c r="C6" t="str">
-        <f t="shared" si="0"/>
+        <f>PROPER(TRIM(A6))</f>
         <v>Moveis_Decoracao</v>
       </c>
       <c r="D6" t="str">
-        <f t="shared" si="1"/>
+        <f>PROPER(TRIM(B6))</f>
         <v>Furniture_Decor</v>
       </c>
     </row>
@@ -1418,11 +1418,11 @@
         <v>13</v>
       </c>
       <c r="C7" t="str">
-        <f t="shared" si="0"/>
+        <f>PROPER(TRIM(A7))</f>
         <v>Esporte_Lazer</v>
       </c>
       <c r="D7" t="str">
-        <f t="shared" si="1"/>
+        <f>PROPER(TRIM(B7))</f>
         <v>Sports_Leisure</v>
       </c>
     </row>
@@ -1434,11 +1434,11 @@
         <v>15</v>
       </c>
       <c r="C8" t="str">
-        <f t="shared" si="0"/>
+        <f>PROPER(TRIM(A8))</f>
         <v>Perfumaria</v>
       </c>
       <c r="D8" t="str">
-        <f t="shared" si="1"/>
+        <f>PROPER(TRIM(B8))</f>
         <v>Perfumery</v>
       </c>
     </row>
@@ -1450,11 +1450,11 @@
         <v>17</v>
       </c>
       <c r="C9" t="str">
-        <f t="shared" si="0"/>
+        <f>PROPER(TRIM(A9))</f>
         <v>Utilidades_Domesticas</v>
       </c>
       <c r="D9" t="str">
-        <f t="shared" si="1"/>
+        <f>PROPER(TRIM(B9))</f>
         <v>Housewares</v>
       </c>
     </row>
@@ -1466,11 +1466,11 @@
         <v>19</v>
       </c>
       <c r="C10" t="str">
-        <f t="shared" si="0"/>
+        <f>PROPER(TRIM(A10))</f>
         <v>Telefonia</v>
       </c>
       <c r="D10" t="str">
-        <f t="shared" si="1"/>
+        <f>PROPER(TRIM(B10))</f>
         <v>Telephony</v>
       </c>
     </row>
@@ -1482,11 +1482,11 @@
         <v>21</v>
       </c>
       <c r="C11" t="str">
-        <f t="shared" si="0"/>
+        <f>PROPER(TRIM(A11))</f>
         <v>Relogios_Presentes</v>
       </c>
       <c r="D11" t="str">
-        <f t="shared" si="1"/>
+        <f>PROPER(TRIM(B11))</f>
         <v>Watches_Gifts</v>
       </c>
     </row>
@@ -1498,11 +1498,11 @@
         <v>23</v>
       </c>
       <c r="C12" t="str">
-        <f t="shared" si="0"/>
+        <f>PROPER(TRIM(A12))</f>
         <v>Alimentos_Bebidas</v>
       </c>
       <c r="D12" t="str">
-        <f t="shared" si="1"/>
+        <f>PROPER(TRIM(B12))</f>
         <v>Food_Drink</v>
       </c>
     </row>
@@ -1514,11 +1514,11 @@
         <v>25</v>
       </c>
       <c r="C13" t="str">
-        <f t="shared" si="0"/>
+        <f>PROPER(TRIM(A13))</f>
         <v>Bebes</v>
       </c>
       <c r="D13" t="str">
-        <f t="shared" si="1"/>
+        <f>PROPER(TRIM(B13))</f>
         <v>Baby</v>
       </c>
     </row>
@@ -1530,11 +1530,11 @@
         <v>27</v>
       </c>
       <c r="C14" t="str">
-        <f t="shared" si="0"/>
+        <f>PROPER(TRIM(A14))</f>
         <v>Papelaria</v>
       </c>
       <c r="D14" t="str">
-        <f t="shared" si="1"/>
+        <f>PROPER(TRIM(B14))</f>
         <v>Stationery</v>
       </c>
     </row>
@@ -1546,11 +1546,11 @@
         <v>29</v>
       </c>
       <c r="C15" t="str">
-        <f t="shared" si="0"/>
+        <f>PROPER(TRIM(A15))</f>
         <v>Tablets_Impressao_Imagem</v>
       </c>
       <c r="D15" t="str">
-        <f t="shared" si="1"/>
+        <f>PROPER(TRIM(B15))</f>
         <v>Tablets_Printing_Image</v>
       </c>
     </row>
@@ -1562,11 +1562,11 @@
         <v>31</v>
       </c>
       <c r="C16" t="str">
-        <f t="shared" si="0"/>
+        <f>PROPER(TRIM(A16))</f>
         <v>Brinquedos</v>
       </c>
       <c r="D16" t="str">
-        <f t="shared" si="1"/>
+        <f>PROPER(TRIM(B16))</f>
         <v>Toys</v>
       </c>
     </row>
@@ -1578,11 +1578,11 @@
         <v>33</v>
       </c>
       <c r="C17" t="str">
-        <f t="shared" si="0"/>
+        <f>PROPER(TRIM(A17))</f>
         <v>Telefonia_Fixa</v>
       </c>
       <c r="D17" t="str">
-        <f t="shared" si="1"/>
+        <f>PROPER(TRIM(B17))</f>
         <v>Fixed_Telephony</v>
       </c>
     </row>
@@ -1594,11 +1594,11 @@
         <v>35</v>
       </c>
       <c r="C18" t="str">
-        <f t="shared" si="0"/>
+        <f>PROPER(TRIM(A18))</f>
         <v>Ferramentas_Jardim</v>
       </c>
       <c r="D18" t="str">
-        <f t="shared" si="1"/>
+        <f>PROPER(TRIM(B18))</f>
         <v>Garden_Tools</v>
       </c>
     </row>
@@ -1610,11 +1610,11 @@
         <v>37</v>
       </c>
       <c r="C19" t="str">
-        <f t="shared" si="0"/>
+        <f>PROPER(TRIM(A19))</f>
         <v>Fashion_Bolsas_E_Acessorios</v>
       </c>
       <c r="D19" t="str">
-        <f t="shared" si="1"/>
+        <f>PROPER(TRIM(B19))</f>
         <v>Fashion_Bags_Accessories</v>
       </c>
     </row>
@@ -1626,11 +1626,11 @@
         <v>39</v>
       </c>
       <c r="C20" t="str">
-        <f t="shared" si="0"/>
+        <f>PROPER(TRIM(A20))</f>
         <v>Eletroportateis</v>
       </c>
       <c r="D20" t="str">
-        <f t="shared" si="1"/>
+        <f>PROPER(TRIM(B20))</f>
         <v>Small_Appliances</v>
       </c>
     </row>
@@ -1642,11 +1642,11 @@
         <v>40</v>
       </c>
       <c r="C21" t="str">
-        <f t="shared" si="0"/>
+        <f>PROPER(TRIM(A21))</f>
         <v>Consoles_Games</v>
       </c>
       <c r="D21" t="str">
-        <f t="shared" si="1"/>
+        <f>PROPER(TRIM(B21))</f>
         <v>Consoles_Games</v>
       </c>
     </row>
@@ -1658,11 +1658,11 @@
         <v>41</v>
       </c>
       <c r="C22" t="str">
-        <f t="shared" si="0"/>
+        <f>PROPER(TRIM(A22))</f>
         <v>Audio</v>
       </c>
       <c r="D22" t="str">
-        <f t="shared" si="1"/>
+        <f>PROPER(TRIM(B22))</f>
         <v>Audio</v>
       </c>
     </row>
@@ -1674,11 +1674,11 @@
         <v>43</v>
       </c>
       <c r="C23" t="str">
-        <f t="shared" si="0"/>
+        <f>PROPER(TRIM(A23))</f>
         <v>Fashion_Calcados</v>
       </c>
       <c r="D23" t="str">
-        <f t="shared" si="1"/>
+        <f>PROPER(TRIM(B23))</f>
         <v>Fashion_Shoes</v>
       </c>
     </row>
@@ -1690,11 +1690,11 @@
         <v>44</v>
       </c>
       <c r="C24" t="str">
-        <f t="shared" si="0"/>
+        <f>PROPER(TRIM(A24))</f>
         <v>Cool_Stuff</v>
       </c>
       <c r="D24" t="str">
-        <f t="shared" si="1"/>
+        <f>PROPER(TRIM(B24))</f>
         <v>Cool_Stuff</v>
       </c>
     </row>
@@ -1706,11 +1706,11 @@
         <v>46</v>
       </c>
       <c r="C25" t="str">
-        <f t="shared" si="0"/>
+        <f>PROPER(TRIM(A25))</f>
         <v>Malas_Acessorios</v>
       </c>
       <c r="D25" t="str">
-        <f t="shared" si="1"/>
+        <f>PROPER(TRIM(B25))</f>
         <v>Luggage_Accessories</v>
       </c>
     </row>
@@ -1722,11 +1722,11 @@
         <v>48</v>
       </c>
       <c r="C26" t="str">
-        <f t="shared" si="0"/>
+        <f>PROPER(TRIM(A26))</f>
         <v>Climatizacao</v>
       </c>
       <c r="D26" t="str">
-        <f t="shared" si="1"/>
+        <f>PROPER(TRIM(B26))</f>
         <v>Air_Conditioning</v>
       </c>
     </row>
@@ -1738,11 +1738,11 @@
         <v>50</v>
       </c>
       <c r="C27" t="str">
-        <f t="shared" si="0"/>
+        <f>PROPER(TRIM(A27))</f>
         <v>Construcao_Ferramentas_Construcao</v>
       </c>
       <c r="D27" t="str">
-        <f t="shared" si="1"/>
+        <f>PROPER(TRIM(B27))</f>
         <v>Construction_Tools_Construction</v>
       </c>
     </row>
@@ -1754,11 +1754,11 @@
         <v>52</v>
       </c>
       <c r="C28" t="str">
-        <f t="shared" si="0"/>
+        <f>PROPER(TRIM(A28))</f>
         <v>Moveis_Cozinha_Area_De_Servico_Jantar_E_Jardim</v>
       </c>
       <c r="D28" t="str">
-        <f t="shared" si="1"/>
+        <f>PROPER(TRIM(B28))</f>
         <v>Kitchen_Dining_Laundry_Garden_Furniture</v>
       </c>
     </row>
@@ -1770,11 +1770,11 @@
         <v>54</v>
       </c>
       <c r="C29" t="str">
-        <f t="shared" si="0"/>
+        <f>PROPER(TRIM(A29))</f>
         <v>Construcao_Ferramentas_Jardim</v>
       </c>
       <c r="D29" t="str">
-        <f t="shared" si="1"/>
+        <f>PROPER(TRIM(B29))</f>
         <v>Costruction_Tools_Garden</v>
       </c>
     </row>
@@ -1786,11 +1786,11 @@
         <v>56</v>
       </c>
       <c r="C30" t="str">
-        <f t="shared" si="0"/>
+        <f>PROPER(TRIM(A30))</f>
         <v>Fashion_Roupa_Masculina</v>
       </c>
       <c r="D30" t="str">
-        <f t="shared" si="1"/>
+        <f>PROPER(TRIM(B30))</f>
         <v>Fashion_Male_Clothing</v>
       </c>
     </row>
@@ -1802,11 +1802,11 @@
         <v>57</v>
       </c>
       <c r="C31" t="str">
-        <f t="shared" si="0"/>
+        <f>PROPER(TRIM(A31))</f>
         <v>Pet_Shop</v>
       </c>
       <c r="D31" t="str">
-        <f t="shared" si="1"/>
+        <f>PROPER(TRIM(B31))</f>
         <v>Pet_Shop</v>
       </c>
     </row>
@@ -1818,11 +1818,11 @@
         <v>59</v>
       </c>
       <c r="C32" t="str">
-        <f t="shared" si="0"/>
+        <f>PROPER(TRIM(A32))</f>
         <v>Moveis_Escritorio</v>
       </c>
       <c r="D32" t="str">
-        <f t="shared" si="1"/>
+        <f>PROPER(TRIM(B32))</f>
         <v>Office_Furniture</v>
       </c>
     </row>
@@ -1834,11 +1834,11 @@
         <v>60</v>
       </c>
       <c r="C33" t="str">
-        <f t="shared" si="0"/>
+        <f>PROPER(TRIM(A33))</f>
         <v>Market_Place</v>
       </c>
       <c r="D33" t="str">
-        <f t="shared" si="1"/>
+        <f>PROPER(TRIM(B33))</f>
         <v>Market_Place</v>
       </c>
     </row>
@@ -1850,11 +1850,11 @@
         <v>62</v>
       </c>
       <c r="C34" t="str">
-        <f t="shared" si="0"/>
+        <f>PROPER(TRIM(A34))</f>
         <v>Eletronicos</v>
       </c>
       <c r="D34" t="str">
-        <f t="shared" si="1"/>
+        <f>PROPER(TRIM(B34))</f>
         <v>Electronics</v>
       </c>
     </row>
@@ -1866,11 +1866,11 @@
         <v>64</v>
       </c>
       <c r="C35" t="str">
-        <f t="shared" si="0"/>
+        <f>PROPER(TRIM(A35))</f>
         <v>Eletrodomesticos</v>
       </c>
       <c r="D35" t="str">
-        <f t="shared" si="1"/>
+        <f>PROPER(TRIM(B35))</f>
         <v>Home_Appliances</v>
       </c>
     </row>
@@ -1882,11 +1882,11 @@
         <v>66</v>
       </c>
       <c r="C36" t="str">
-        <f t="shared" si="0"/>
+        <f>PROPER(TRIM(A36))</f>
         <v>Artigos_De_Festas</v>
       </c>
       <c r="D36" t="str">
-        <f t="shared" si="1"/>
+        <f>PROPER(TRIM(B36))</f>
         <v>Party_Supplies</v>
       </c>
     </row>
@@ -1898,11 +1898,11 @@
         <v>68</v>
       </c>
       <c r="C37" t="str">
-        <f t="shared" si="0"/>
+        <f>PROPER(TRIM(A37))</f>
         <v>Casa_Conforto</v>
       </c>
       <c r="D37" t="str">
-        <f t="shared" si="1"/>
+        <f>PROPER(TRIM(B37))</f>
         <v>Home_Confort</v>
       </c>
     </row>
@@ -1914,11 +1914,11 @@
         <v>70</v>
       </c>
       <c r="C38" t="str">
-        <f t="shared" si="0"/>
+        <f>PROPER(TRIM(A38))</f>
         <v>Construcao_Ferramentas_Ferramentas</v>
       </c>
       <c r="D38" t="str">
-        <f t="shared" si="1"/>
+        <f>PROPER(TRIM(B38))</f>
         <v>Costruction_Tools_Tools</v>
       </c>
     </row>
@@ -1930,11 +1930,11 @@
         <v>72</v>
       </c>
       <c r="C39" t="str">
-        <f t="shared" si="0"/>
+        <f>PROPER(TRIM(A39))</f>
         <v>Agro_Industria_E_Comercio</v>
       </c>
       <c r="D39" t="str">
-        <f t="shared" si="1"/>
+        <f>PROPER(TRIM(B39))</f>
         <v>Agro_Industry_And_Commerce</v>
       </c>
     </row>
@@ -1946,11 +1946,11 @@
         <v>74</v>
       </c>
       <c r="C40" t="str">
-        <f t="shared" si="0"/>
+        <f>PROPER(TRIM(A40))</f>
         <v>Moveis_Colchao_E_Estofado</v>
       </c>
       <c r="D40" t="str">
-        <f t="shared" si="1"/>
+        <f>PROPER(TRIM(B40))</f>
         <v>Furniture_Mattress_And_Upholstery</v>
       </c>
     </row>
@@ -1962,11 +1962,11 @@
         <v>76</v>
       </c>
       <c r="C41" t="str">
-        <f t="shared" si="0"/>
+        <f>PROPER(TRIM(A41))</f>
         <v>Livros_Tecnicos</v>
       </c>
       <c r="D41" t="str">
-        <f t="shared" si="1"/>
+        <f>PROPER(TRIM(B41))</f>
         <v>Books_Technical</v>
       </c>
     </row>
@@ -1978,11 +1978,11 @@
         <v>78</v>
       </c>
       <c r="C42" t="str">
-        <f t="shared" si="0"/>
+        <f>PROPER(TRIM(A42))</f>
         <v>Casa_Construcao</v>
       </c>
       <c r="D42" t="str">
-        <f t="shared" si="1"/>
+        <f>PROPER(TRIM(B42))</f>
         <v>Home_Construction</v>
       </c>
     </row>
@@ -1994,11 +1994,11 @@
         <v>80</v>
       </c>
       <c r="C43" t="str">
-        <f t="shared" si="0"/>
+        <f>PROPER(TRIM(A43))</f>
         <v>Instrumentos_Musicais</v>
       </c>
       <c r="D43" t="str">
-        <f t="shared" si="1"/>
+        <f>PROPER(TRIM(B43))</f>
         <v>Musical_Instruments</v>
       </c>
     </row>
@@ -2010,11 +2010,11 @@
         <v>82</v>
       </c>
       <c r="C44" t="str">
-        <f t="shared" si="0"/>
+        <f>PROPER(TRIM(A44))</f>
         <v>Moveis_Sala</v>
       </c>
       <c r="D44" t="str">
-        <f t="shared" si="1"/>
+        <f>PROPER(TRIM(B44))</f>
         <v>Furniture_Living_Room</v>
       </c>
     </row>
@@ -2026,11 +2026,11 @@
         <v>84</v>
       </c>
       <c r="C45" t="str">
-        <f t="shared" si="0"/>
+        <f>PROPER(TRIM(A45))</f>
         <v>Construcao_Ferramentas_Iluminacao</v>
       </c>
       <c r="D45" t="str">
-        <f t="shared" si="1"/>
+        <f>PROPER(TRIM(B45))</f>
         <v>Construction_Tools_Lights</v>
       </c>
     </row>
@@ -2042,11 +2042,11 @@
         <v>86</v>
       </c>
       <c r="C46" t="str">
-        <f t="shared" si="0"/>
+        <f>PROPER(TRIM(A46))</f>
         <v>Industria_Comercio_E_Negocios</v>
       </c>
       <c r="D46" t="str">
-        <f t="shared" si="1"/>
+        <f>PROPER(TRIM(B46))</f>
         <v>Industry_Commerce_And_Business</v>
       </c>
     </row>
@@ -2058,11 +2058,11 @@
         <v>88</v>
       </c>
       <c r="C47" t="str">
-        <f t="shared" si="0"/>
+        <f>PROPER(TRIM(A47))</f>
         <v>Alimentos</v>
       </c>
       <c r="D47" t="str">
-        <f t="shared" si="1"/>
+        <f>PROPER(TRIM(B47))</f>
         <v>Food</v>
       </c>
     </row>
@@ -2074,11 +2074,11 @@
         <v>90</v>
       </c>
       <c r="C48" t="str">
-        <f t="shared" si="0"/>
+        <f>PROPER(TRIM(A48))</f>
         <v>Artes</v>
       </c>
       <c r="D48" t="str">
-        <f t="shared" si="1"/>
+        <f>PROPER(TRIM(B48))</f>
         <v>Art</v>
       </c>
     </row>
@@ -2090,11 +2090,11 @@
         <v>92</v>
       </c>
       <c r="C49" t="str">
-        <f t="shared" si="0"/>
+        <f>PROPER(TRIM(A49))</f>
         <v>Moveis_Quarto</v>
       </c>
       <c r="D49" t="str">
-        <f t="shared" si="1"/>
+        <f>PROPER(TRIM(B49))</f>
         <v>Furniture_Bedroom</v>
       </c>
     </row>
@@ -2106,11 +2106,11 @@
         <v>94</v>
       </c>
       <c r="C50" t="str">
-        <f t="shared" si="0"/>
+        <f>PROPER(TRIM(A50))</f>
         <v>Livros_Interesse_Geral</v>
       </c>
       <c r="D50" t="str">
-        <f t="shared" si="1"/>
+        <f>PROPER(TRIM(B50))</f>
         <v>Books_General_Interest</v>
       </c>
     </row>
@@ -2122,11 +2122,11 @@
         <v>96</v>
       </c>
       <c r="C51" t="str">
-        <f t="shared" si="0"/>
+        <f>PROPER(TRIM(A51))</f>
         <v>Construcao_Ferramentas_Seguranca</v>
       </c>
       <c r="D51" t="str">
-        <f t="shared" si="1"/>
+        <f>PROPER(TRIM(B51))</f>
         <v>Construction_Tools_Safety</v>
       </c>
     </row>
@@ -2138,11 +2138,11 @@
         <v>98</v>
       </c>
       <c r="C52" t="str">
-        <f t="shared" si="0"/>
+        <f>PROPER(TRIM(A52))</f>
         <v>Fashion_Underwear_E_Moda_Praia</v>
       </c>
       <c r="D52" t="str">
-        <f t="shared" si="1"/>
+        <f>PROPER(TRIM(B52))</f>
         <v>Fashion_Underwear_Beach</v>
       </c>
     </row>
@@ -2154,11 +2154,11 @@
         <v>100</v>
       </c>
       <c r="C53" t="str">
-        <f t="shared" si="0"/>
+        <f>PROPER(TRIM(A53))</f>
         <v>Fashion_Esporte</v>
       </c>
       <c r="D53" t="str">
-        <f t="shared" si="1"/>
+        <f>PROPER(TRIM(B53))</f>
         <v>Fashion_Sport</v>
       </c>
     </row>
@@ -2170,11 +2170,11 @@
         <v>102</v>
       </c>
       <c r="C54" t="str">
-        <f t="shared" si="0"/>
+        <f>PROPER(TRIM(A54))</f>
         <v>Sinalizacao_E_Seguranca</v>
       </c>
       <c r="D54" t="str">
-        <f t="shared" si="1"/>
+        <f>PROPER(TRIM(B54))</f>
         <v>Signaling_And_Security</v>
       </c>
     </row>
@@ -2186,11 +2186,11 @@
         <v>104</v>
       </c>
       <c r="C55" t="str">
-        <f t="shared" si="0"/>
+        <f>PROPER(TRIM(A55))</f>
         <v>Pcs</v>
       </c>
       <c r="D55" t="str">
-        <f t="shared" si="1"/>
+        <f>PROPER(TRIM(B55))</f>
         <v>Computers</v>
       </c>
     </row>
@@ -2202,11 +2202,11 @@
         <v>106</v>
       </c>
       <c r="C56" t="str">
-        <f t="shared" si="0"/>
+        <f>PROPER(TRIM(A56))</f>
         <v>Artigos_De_Natal</v>
       </c>
       <c r="D56" t="str">
-        <f t="shared" si="1"/>
+        <f>PROPER(TRIM(B56))</f>
         <v>Christmas_Supplies</v>
       </c>
     </row>
@@ -2218,11 +2218,11 @@
         <v>108</v>
       </c>
       <c r="C57" t="str">
-        <f t="shared" si="0"/>
+        <f>PROPER(TRIM(A57))</f>
         <v>Fashion_Roupa_Feminina</v>
       </c>
       <c r="D57" t="str">
-        <f t="shared" si="1"/>
+        <f>PROPER(TRIM(B57))</f>
         <v>Fashio_Female_Clothing</v>
       </c>
     </row>
@@ -2234,11 +2234,11 @@
         <v>110</v>
       </c>
       <c r="C58" t="str">
-        <f t="shared" si="0"/>
+        <f>PROPER(TRIM(A58))</f>
         <v>Eletrodomesticos_2</v>
       </c>
       <c r="D58" t="str">
-        <f t="shared" si="1"/>
+        <f>PROPER(TRIM(B58))</f>
         <v>Home_Appliances_2</v>
       </c>
     </row>
@@ -2250,11 +2250,11 @@
         <v>112</v>
       </c>
       <c r="C59" t="str">
-        <f t="shared" si="0"/>
+        <f>PROPER(TRIM(A59))</f>
         <v>Livros_Importados</v>
       </c>
       <c r="D59" t="str">
-        <f t="shared" si="1"/>
+        <f>PROPER(TRIM(B59))</f>
         <v>Books_Imported</v>
       </c>
     </row>
@@ -2266,11 +2266,11 @@
         <v>114</v>
       </c>
       <c r="C60" t="str">
-        <f t="shared" si="0"/>
+        <f>PROPER(TRIM(A60))</f>
         <v>Bebidas</v>
       </c>
       <c r="D60" t="str">
-        <f t="shared" si="1"/>
+        <f>PROPER(TRIM(B60))</f>
         <v>Drinks</v>
       </c>
     </row>
@@ -2282,11 +2282,11 @@
         <v>116</v>
       </c>
       <c r="C61" t="str">
-        <f t="shared" si="0"/>
+        <f>PROPER(TRIM(A61))</f>
         <v>Cine_Foto</v>
       </c>
       <c r="D61" t="str">
-        <f t="shared" si="1"/>
+        <f>PROPER(TRIM(B61))</f>
         <v>Cine_Photo</v>
       </c>
     </row>
@@ -2298,11 +2298,11 @@
         <v>117</v>
       </c>
       <c r="C62" t="str">
-        <f t="shared" si="0"/>
+        <f>PROPER(TRIM(A62))</f>
         <v>La_Cuisine</v>
       </c>
       <c r="D62" t="str">
-        <f t="shared" si="1"/>
+        <f>PROPER(TRIM(B62))</f>
         <v>La_Cuisine</v>
       </c>
     </row>
@@ -2314,11 +2314,11 @@
         <v>119</v>
       </c>
       <c r="C63" t="str">
-        <f t="shared" si="0"/>
+        <f>PROPER(TRIM(A63))</f>
         <v>Musica</v>
       </c>
       <c r="D63" t="str">
-        <f t="shared" si="1"/>
+        <f>PROPER(TRIM(B63))</f>
         <v>Music</v>
       </c>
     </row>
@@ -2330,11 +2330,11 @@
         <v>121</v>
       </c>
       <c r="C64" t="str">
-        <f t="shared" si="0"/>
+        <f>PROPER(TRIM(A64))</f>
         <v>Casa_Conforto_2</v>
       </c>
       <c r="D64" t="str">
-        <f t="shared" si="1"/>
+        <f>PROPER(TRIM(B64))</f>
         <v>Home_Comfort_2</v>
       </c>
     </row>
@@ -2346,11 +2346,11 @@
         <v>123</v>
       </c>
       <c r="C65" t="str">
-        <f t="shared" si="0"/>
+        <f>PROPER(TRIM(A65))</f>
         <v>Portateis_Casa_Forno_E_Cafe</v>
       </c>
       <c r="D65" t="str">
-        <f t="shared" si="1"/>
+        <f>PROPER(TRIM(B65))</f>
         <v>Small_Appliances_Home_Oven_And_Coffee</v>
       </c>
     </row>
@@ -2362,11 +2362,11 @@
         <v>125</v>
       </c>
       <c r="C66" t="str">
-        <f t="shared" ref="C66:C72" si="2">PROPER(TRIM(A66))</f>
+        <f>PROPER(TRIM(A66))</f>
         <v>Cds_Dvds_Musicais</v>
       </c>
       <c r="D66" t="str">
-        <f t="shared" ref="D66:D72" si="3">PROPER(TRIM(B66))</f>
+        <f>PROPER(TRIM(B66))</f>
         <v>Cds_Dvds_Musicals</v>
       </c>
     </row>
@@ -2378,11 +2378,11 @@
         <v>126</v>
       </c>
       <c r="C67" t="str">
-        <f t="shared" si="2"/>
+        <f>PROPER(TRIM(A67))</f>
         <v>Dvds_Blu_Ray</v>
       </c>
       <c r="D67" t="str">
-        <f t="shared" si="3"/>
+        <f>PROPER(TRIM(B67))</f>
         <v>Dvds_Blu_Ray</v>
       </c>
     </row>
@@ -2394,11 +2394,11 @@
         <v>128</v>
       </c>
       <c r="C68" t="str">
-        <f t="shared" si="2"/>
+        <f>PROPER(TRIM(A68))</f>
         <v>Flores</v>
       </c>
       <c r="D68" t="str">
-        <f t="shared" si="3"/>
+        <f>PROPER(TRIM(B68))</f>
         <v>Flowers</v>
       </c>
     </row>
@@ -2410,11 +2410,11 @@
         <v>130</v>
       </c>
       <c r="C69" t="str">
-        <f t="shared" si="2"/>
+        <f>PROPER(TRIM(A69))</f>
         <v>Artes_E_Artesanato</v>
       </c>
       <c r="D69" t="str">
-        <f t="shared" si="3"/>
+        <f>PROPER(TRIM(B69))</f>
         <v>Arts_And_Craftmanship</v>
       </c>
     </row>
@@ -2426,11 +2426,11 @@
         <v>132</v>
       </c>
       <c r="C70" t="str">
-        <f t="shared" si="2"/>
+        <f>PROPER(TRIM(A70))</f>
         <v>Fraldas_Higiene</v>
       </c>
       <c r="D70" t="str">
-        <f t="shared" si="3"/>
+        <f>PROPER(TRIM(B70))</f>
         <v>Diapers_And_Hygiene</v>
       </c>
     </row>
@@ -2442,11 +2442,11 @@
         <v>134</v>
       </c>
       <c r="C71" t="str">
-        <f t="shared" si="2"/>
+        <f>PROPER(TRIM(A71))</f>
         <v>Fashion_Roupa_Infanto_Juvenil</v>
       </c>
       <c r="D71" t="str">
-        <f t="shared" si="3"/>
+        <f>PROPER(TRIM(B71))</f>
         <v>Fashion_Childrens_Clothes</v>
       </c>
     </row>
@@ -2458,11 +2458,11 @@
         <v>136</v>
       </c>
       <c r="C72" t="str">
-        <f t="shared" si="2"/>
+        <f>PROPER(TRIM(A72))</f>
         <v>Seguros_E_Servicos</v>
       </c>
       <c r="D72" t="str">
-        <f t="shared" si="3"/>
+        <f>PROPER(TRIM(B72))</f>
         <v>Security_And_Services</v>
       </c>
     </row>

</xml_diff>